<commit_message>
feat: complete 1.4.1 import and mapping updates
</commit_message>
<xml_diff>
--- a/assets/币种映射表.xlsx
+++ b/assets/币种映射表.xlsx
@@ -7,7 +7,7 @@
     <workbookView windowHeight="17240"/>
   </bookViews>
   <sheets>
-    <sheet name="balance" sheetId="2" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="3" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,15 +27,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="142">
-  <si>
-    <t>简体中文简称</t>
-  </si>
-  <si>
-    <t xml:space="preserve">繁体中文简称 </t>
-  </si>
-  <si>
-    <t>英文简称</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="424">
+  <si>
+    <t>简体中文简称 (A列)</t>
+  </si>
+  <si>
+    <t>繁体中文简称 (B列)</t>
+  </si>
+  <si>
+    <t>英文简称/代码 (C列)</t>
   </si>
   <si>
     <t>人民币</t>
@@ -92,27 +92,18 @@
     <t>港元</t>
   </si>
   <si>
-    <t>港元 / 港幣</t>
-  </si>
-  <si>
     <t>HKD</t>
   </si>
   <si>
     <t>澳元</t>
   </si>
   <si>
-    <t>澳元 / 澳幣</t>
-  </si>
-  <si>
     <t>AUD</t>
   </si>
   <si>
     <t>加元</t>
   </si>
   <si>
-    <t>加元 / 加幣</t>
-  </si>
-  <si>
     <t>CAD</t>
   </si>
   <si>
@@ -122,15 +113,30 @@
     <t>CHF</t>
   </si>
   <si>
-    <t>新币 / 新加坡元</t>
-  </si>
-  <si>
-    <t>新幣 / 新加坡元</t>
+    <t>新加坡元</t>
   </si>
   <si>
     <t>SGD</t>
   </si>
   <si>
+    <t>新台币</t>
+  </si>
+  <si>
+    <t>新台幣</t>
+  </si>
+  <si>
+    <t>TWD</t>
+  </si>
+  <si>
+    <t>韩元</t>
+  </si>
+  <si>
+    <t>韓元</t>
+  </si>
+  <si>
+    <t>KRW</t>
+  </si>
+  <si>
     <t>纽元 / 新西兰元</t>
   </si>
   <si>
@@ -140,97 +146,511 @@
     <t>NZD</t>
   </si>
   <si>
-    <t>韩元</t>
-  </si>
-  <si>
-    <t>韓元 / 韓圜</t>
-  </si>
-  <si>
-    <t>KRW</t>
-  </si>
-  <si>
-    <t>新台币</t>
-  </si>
-  <si>
-    <t>新台幣</t>
-  </si>
-  <si>
-    <t>TWD</t>
-  </si>
-  <si>
     <t>澳门元</t>
   </si>
   <si>
-    <t>澳門元 / 澳門幣</t>
+    <t>澳門元</t>
   </si>
   <si>
     <t>MOP</t>
   </si>
   <si>
-    <t>卢布 / 俄罗斯卢布</t>
-  </si>
-  <si>
-    <t>盧布 / 俄羅斯盧布</t>
+    <t>瑞典克朗</t>
+  </si>
+  <si>
+    <t>SEK</t>
+  </si>
+  <si>
+    <t>挪威克朗</t>
+  </si>
+  <si>
+    <t>NOK</t>
+  </si>
+  <si>
+    <t>丹麦克朗</t>
+  </si>
+  <si>
+    <t>丹麥克朗</t>
+  </si>
+  <si>
+    <t>DKK</t>
+  </si>
+  <si>
+    <t>冰岛克朗</t>
+  </si>
+  <si>
+    <t>冰島克朗</t>
+  </si>
+  <si>
+    <t>ISK</t>
+  </si>
+  <si>
+    <t>泰铢</t>
+  </si>
+  <si>
+    <t>泰銖</t>
+  </si>
+  <si>
+    <t>THB</t>
+  </si>
+  <si>
+    <t>林吉特 / 马币</t>
+  </si>
+  <si>
+    <t>林吉特 / 馬幣</t>
+  </si>
+  <si>
+    <t>MYR</t>
+  </si>
+  <si>
+    <t>印尼盾</t>
+  </si>
+  <si>
+    <t>IDR</t>
+  </si>
+  <si>
+    <t>菲律宾比索</t>
+  </si>
+  <si>
+    <t>菲律賓比索</t>
+  </si>
+  <si>
+    <t>PHP</t>
+  </si>
+  <si>
+    <t>越南盾</t>
+  </si>
+  <si>
+    <t>VND</t>
+  </si>
+  <si>
+    <t>印度卢比</t>
+  </si>
+  <si>
+    <t>印度盧比</t>
+  </si>
+  <si>
+    <t>INR</t>
+  </si>
+  <si>
+    <t>巴基斯坦卢比</t>
+  </si>
+  <si>
+    <t>巴基斯坦盧比</t>
+  </si>
+  <si>
+    <t>PKR</t>
+  </si>
+  <si>
+    <t>斯里兰卡卢比</t>
+  </si>
+  <si>
+    <t>斯里蘭卡盧比</t>
+  </si>
+  <si>
+    <t>LKR</t>
+  </si>
+  <si>
+    <t>尼泊尔卢比</t>
+  </si>
+  <si>
+    <t>尼泊爾盧比</t>
+  </si>
+  <si>
+    <t>NPR</t>
+  </si>
+  <si>
+    <t>孟加拉塔卡</t>
+  </si>
+  <si>
+    <t>BDT</t>
+  </si>
+  <si>
+    <t>缅甸元</t>
+  </si>
+  <si>
+    <t>緬甸元</t>
+  </si>
+  <si>
+    <t>MMK</t>
+  </si>
+  <si>
+    <t>瑞尔 (柬埔寨)</t>
+  </si>
+  <si>
+    <t>瑞爾 (柬埔寨)</t>
+  </si>
+  <si>
+    <t>KHR</t>
+  </si>
+  <si>
+    <t>基普 (老挝)</t>
+  </si>
+  <si>
+    <t>基普 (老撾)</t>
+  </si>
+  <si>
+    <t>LAK</t>
+  </si>
+  <si>
+    <t>图格里克 (蒙古)</t>
+  </si>
+  <si>
+    <t>圖格里克 (蒙古)</t>
+  </si>
+  <si>
+    <t>MNT</t>
+  </si>
+  <si>
+    <t>索姆 (乌兹别克斯坦)</t>
+  </si>
+  <si>
+    <t>索姆 (烏茲別克斯坦)</t>
+  </si>
+  <si>
+    <t>UZS</t>
+  </si>
+  <si>
+    <t>吉尔吉斯斯坦索姆</t>
+  </si>
+  <si>
+    <t>吉爾吉斯斯坦索姆</t>
+  </si>
+  <si>
+    <t>KGS</t>
+  </si>
+  <si>
+    <t>塔吉克斯坦索莫尼</t>
+  </si>
+  <si>
+    <t>TJS</t>
+  </si>
+  <si>
+    <t>坚戈 (哈萨克斯坦)</t>
+  </si>
+  <si>
+    <t>堅戈 (哈薩克斯坦)</t>
+  </si>
+  <si>
+    <t>KZT</t>
+  </si>
+  <si>
+    <t>阿富汗尼</t>
+  </si>
+  <si>
+    <t>AFN</t>
+  </si>
+  <si>
+    <t>巴西雷亚尔</t>
+  </si>
+  <si>
+    <t>巴西雷亞爾</t>
+  </si>
+  <si>
+    <t>BRL</t>
+  </si>
+  <si>
+    <t>墨西哥比索</t>
+  </si>
+  <si>
+    <t>MXN</t>
+  </si>
+  <si>
+    <t>阿根廷比索</t>
+  </si>
+  <si>
+    <t>ARS</t>
+  </si>
+  <si>
+    <t>智利比索</t>
+  </si>
+  <si>
+    <t>CLP</t>
+  </si>
+  <si>
+    <t>哥伦比亚比索</t>
+  </si>
+  <si>
+    <t>哥倫比亞比索</t>
+  </si>
+  <si>
+    <t>COP</t>
+  </si>
+  <si>
+    <t>秘鲁索尔</t>
+  </si>
+  <si>
+    <t>秘魯索爾</t>
+  </si>
+  <si>
+    <t>PEN</t>
+  </si>
+  <si>
+    <t>乌拉圭比索</t>
+  </si>
+  <si>
+    <t>烏拉圭比索</t>
+  </si>
+  <si>
+    <t>UYU</t>
+  </si>
+  <si>
+    <t>委内瑞拉玻利瓦尔</t>
+  </si>
+  <si>
+    <t>委內瑞拉玻利瓦爾</t>
+  </si>
+  <si>
+    <t>VES</t>
+  </si>
+  <si>
+    <t>玻利维亚诺</t>
+  </si>
+  <si>
+    <t>玻利維亞諾</t>
+  </si>
+  <si>
+    <t>BOB</t>
+  </si>
+  <si>
+    <t>圭亚那元</t>
+  </si>
+  <si>
+    <t>圭亞那元</t>
+  </si>
+  <si>
+    <t>GYD</t>
+  </si>
+  <si>
+    <t>巴拉圭瓜拉尼</t>
+  </si>
+  <si>
+    <t>PYG</t>
+  </si>
+  <si>
+    <t>苏里南元</t>
+  </si>
+  <si>
+    <t>蘇里南元</t>
+  </si>
+  <si>
+    <t>SRD</t>
+  </si>
+  <si>
+    <t>俄罗斯卢布</t>
+  </si>
+  <si>
+    <t>俄羅斯盧布</t>
   </si>
   <si>
     <t>RUB</t>
   </si>
   <si>
-    <t>印度卢比</t>
-  </si>
-  <si>
-    <t>印度盧比</t>
-  </si>
-  <si>
-    <t>INR</t>
-  </si>
-  <si>
-    <t>泰铢</t>
-  </si>
-  <si>
-    <t>泰銖</t>
-  </si>
-  <si>
-    <t>THB</t>
-  </si>
-  <si>
-    <t>林吉特 / 马币</t>
-  </si>
-  <si>
-    <t>林吉特 / 馬幣</t>
-  </si>
-  <si>
-    <t>MYR</t>
-  </si>
-  <si>
-    <t>印尼盾</t>
-  </si>
-  <si>
-    <t>IDR</t>
-  </si>
-  <si>
-    <t>菲律宾比索</t>
-  </si>
-  <si>
-    <t>菲律賓比索</t>
-  </si>
-  <si>
-    <t>PHP</t>
-  </si>
-  <si>
-    <t>越南盾</t>
-  </si>
-  <si>
-    <t>VND</t>
-  </si>
-  <si>
-    <t>巴西雷亚尔</t>
-  </si>
-  <si>
-    <t>巴西雷亞爾</t>
-  </si>
-  <si>
-    <t>BRL</t>
+    <t>白俄罗斯卢布</t>
+  </si>
+  <si>
+    <t>白俄羅斯盧布</t>
+  </si>
+  <si>
+    <t>BYN</t>
+  </si>
+  <si>
+    <t>乌克兰格里夫纳</t>
+  </si>
+  <si>
+    <t>烏克蘭格里夫納</t>
+  </si>
+  <si>
+    <t>UAH</t>
+  </si>
+  <si>
+    <t>波兰兹罗提</t>
+  </si>
+  <si>
+    <t>波蘭茲羅提</t>
+  </si>
+  <si>
+    <t>PLN</t>
+  </si>
+  <si>
+    <t>匈牙利福林</t>
+  </si>
+  <si>
+    <t>HUF</t>
+  </si>
+  <si>
+    <t>捷克克朗</t>
+  </si>
+  <si>
+    <t>CZK</t>
+  </si>
+  <si>
+    <t>罗马尼亚列伊</t>
+  </si>
+  <si>
+    <t>羅馬尼亞列伊</t>
+  </si>
+  <si>
+    <t>RON</t>
+  </si>
+  <si>
+    <t>塞尔维亚第纳尔</t>
+  </si>
+  <si>
+    <t>塞爾維亞第納爾</t>
+  </si>
+  <si>
+    <t>RSD</t>
+  </si>
+  <si>
+    <t>保加利亚列弗</t>
+  </si>
+  <si>
+    <t>保加利亞列弗</t>
+  </si>
+  <si>
+    <t>BGN</t>
+  </si>
+  <si>
+    <t>阿尔巴尼亚列克</t>
+  </si>
+  <si>
+    <t>阿爾巴尼亞列克</t>
+  </si>
+  <si>
+    <t>ALL</t>
+  </si>
+  <si>
+    <t>波斯尼亚马克</t>
+  </si>
+  <si>
+    <t>波斯尼亞馬克</t>
+  </si>
+  <si>
+    <t>BAM</t>
+  </si>
+  <si>
+    <t>摩尔多瓦列伊</t>
+  </si>
+  <si>
+    <t>摩爾多瓦列伊</t>
+  </si>
+  <si>
+    <t>MDL</t>
+  </si>
+  <si>
+    <t>格鲁吉亚拉里</t>
+  </si>
+  <si>
+    <t>格魯吉亞拉里</t>
+  </si>
+  <si>
+    <t>GEL</t>
+  </si>
+  <si>
+    <t>阿塞拜疆马纳特</t>
+  </si>
+  <si>
+    <t>阿塞拜疆馬納特</t>
+  </si>
+  <si>
+    <t>AZN</t>
+  </si>
+  <si>
+    <t>土耳其里拉</t>
+  </si>
+  <si>
+    <t>TRY</t>
+  </si>
+  <si>
+    <t>阿联酋迪拉姆</t>
+  </si>
+  <si>
+    <t>阿聯酋迪拉姆</t>
+  </si>
+  <si>
+    <t>AED</t>
+  </si>
+  <si>
+    <t>沙特里亚尔</t>
+  </si>
+  <si>
+    <t>沙特里亞爾</t>
+  </si>
+  <si>
+    <t>SAR</t>
+  </si>
+  <si>
+    <t>以色列新谢克尔</t>
+  </si>
+  <si>
+    <t>以色列新謝克爾</t>
+  </si>
+  <si>
+    <t>ILS</t>
+  </si>
+  <si>
+    <t>卡塔尔里亚尔</t>
+  </si>
+  <si>
+    <t>卡塔爾里亞爾</t>
+  </si>
+  <si>
+    <t>QAR</t>
+  </si>
+  <si>
+    <t>科威特第纳尔</t>
+  </si>
+  <si>
+    <t>科威特第納爾</t>
+  </si>
+  <si>
+    <t>KWD</t>
+  </si>
+  <si>
+    <t>巴林第纳尔</t>
+  </si>
+  <si>
+    <t>巴林第納爾</t>
+  </si>
+  <si>
+    <t>BHD</t>
+  </si>
+  <si>
+    <t>阿曼里亚尔</t>
+  </si>
+  <si>
+    <t>阿曼里亞爾</t>
+  </si>
+  <si>
+    <t>OMR</t>
+  </si>
+  <si>
+    <t>约旦第纳尔</t>
+  </si>
+  <si>
+    <t>約旦第納爾</t>
+  </si>
+  <si>
+    <t>JOD</t>
+  </si>
+  <si>
+    <t>黎巴嫩镑</t>
+  </si>
+  <si>
+    <t>黎巴嫩鎊</t>
+  </si>
+  <si>
+    <t>LBP</t>
+  </si>
+  <si>
+    <t>埃及镑</t>
+  </si>
+  <si>
+    <t>埃及鎊</t>
+  </si>
+  <si>
+    <t>EGP</t>
   </si>
   <si>
     <t>南非兰特</t>
@@ -242,186 +662,6 @@
     <t>ZAR</t>
   </si>
   <si>
-    <t>墨西哥比索</t>
-  </si>
-  <si>
-    <t>MXN</t>
-  </si>
-  <si>
-    <t>瑞典克朗</t>
-  </si>
-  <si>
-    <t>SEK</t>
-  </si>
-  <si>
-    <t>挪威克朗</t>
-  </si>
-  <si>
-    <t>NOK</t>
-  </si>
-  <si>
-    <t>丹麦克朗</t>
-  </si>
-  <si>
-    <t>丹麥克朗</t>
-  </si>
-  <si>
-    <t>DKK</t>
-  </si>
-  <si>
-    <t>土耳其里拉</t>
-  </si>
-  <si>
-    <t>TRY</t>
-  </si>
-  <si>
-    <t>阿联酋迪拉姆</t>
-  </si>
-  <si>
-    <t>阿聯酋迪拉姆</t>
-  </si>
-  <si>
-    <t>AED</t>
-  </si>
-  <si>
-    <t>沙特里亚尔</t>
-  </si>
-  <si>
-    <t>沙特里亞爾</t>
-  </si>
-  <si>
-    <t>SAR</t>
-  </si>
-  <si>
-    <t>以色列新谢克尔</t>
-  </si>
-  <si>
-    <t>以色列新謝克爾</t>
-  </si>
-  <si>
-    <t>ILS</t>
-  </si>
-  <si>
-    <t>阿根廷比索</t>
-  </si>
-  <si>
-    <t>ARS</t>
-  </si>
-  <si>
-    <t>智利比索</t>
-  </si>
-  <si>
-    <t>CLP</t>
-  </si>
-  <si>
-    <t>哥伦比亚比索</t>
-  </si>
-  <si>
-    <t>哥倫比亞比索</t>
-  </si>
-  <si>
-    <t>COP</t>
-  </si>
-  <si>
-    <t>秘鲁索尔</t>
-  </si>
-  <si>
-    <t>秘魯索爾</t>
-  </si>
-  <si>
-    <t>PEN</t>
-  </si>
-  <si>
-    <t>埃及镑</t>
-  </si>
-  <si>
-    <t>埃及鎊</t>
-  </si>
-  <si>
-    <t>EGP</t>
-  </si>
-  <si>
-    <t>波兰兹罗提</t>
-  </si>
-  <si>
-    <t>波蘭茲羅提</t>
-  </si>
-  <si>
-    <t>PLN</t>
-  </si>
-  <si>
-    <t>匈牙利福林</t>
-  </si>
-  <si>
-    <t>HUF</t>
-  </si>
-  <si>
-    <t>捷克克朗</t>
-  </si>
-  <si>
-    <t>CZK</t>
-  </si>
-  <si>
-    <t>罗马尼亚列伊</t>
-  </si>
-  <si>
-    <t>羅馬尼亞列伊</t>
-  </si>
-  <si>
-    <t>RON</t>
-  </si>
-  <si>
-    <t>巴基斯坦卢比</t>
-  </si>
-  <si>
-    <t>巴基斯坦盧比</t>
-  </si>
-  <si>
-    <t>PKR</t>
-  </si>
-  <si>
-    <t>孟加拉塔卡</t>
-  </si>
-  <si>
-    <t>BDT</t>
-  </si>
-  <si>
-    <t>斯里兰卡卢比</t>
-  </si>
-  <si>
-    <t>斯里蘭卡盧比</t>
-  </si>
-  <si>
-    <t>LKR</t>
-  </si>
-  <si>
-    <t>哈萨克斯坦坚戈</t>
-  </si>
-  <si>
-    <t>哈薩克斯坦堅戈</t>
-  </si>
-  <si>
-    <t>KZT</t>
-  </si>
-  <si>
-    <t>卡塔尔里亚尔</t>
-  </si>
-  <si>
-    <t>卡塔爾里亞爾</t>
-  </si>
-  <si>
-    <t>QAR</t>
-  </si>
-  <si>
-    <t>科威特第纳尔</t>
-  </si>
-  <si>
-    <t>科威特第納爾</t>
-  </si>
-  <si>
-    <t>KWD</t>
-  </si>
-  <si>
     <t>尼日利亚奈拉</t>
   </si>
   <si>
@@ -440,33 +680,638 @@
     <t>KES</t>
   </si>
   <si>
+    <t>埃塞俄比亚比尔</t>
+  </si>
+  <si>
+    <t>埃塞俄比亞比爾</t>
+  </si>
+  <si>
+    <t>ETB</t>
+  </si>
+  <si>
     <t>摩洛哥迪拉姆</t>
   </si>
   <si>
     <t>MAD</t>
   </si>
   <si>
-    <t>缅甸元</t>
-  </si>
-  <si>
-    <t>緬甸元</t>
-  </si>
-  <si>
-    <t>MMK</t>
+    <t>阿尔及利亚第纳尔</t>
+  </si>
+  <si>
+    <t>阿爾及利亞第納爾</t>
+  </si>
+  <si>
+    <t>DZD</t>
+  </si>
+  <si>
+    <t>安哥拉宽扎</t>
+  </si>
+  <si>
+    <t>安哥拉寬扎</t>
+  </si>
+  <si>
+    <t>AOA</t>
+  </si>
+  <si>
+    <t>普拉</t>
+  </si>
+  <si>
+    <t>BWP</t>
+  </si>
+  <si>
+    <t>布隆迪法郎</t>
+  </si>
+  <si>
+    <t>BIF</t>
+  </si>
+  <si>
+    <t>佛得角埃斯库多</t>
+  </si>
+  <si>
+    <t>佛得角埃斯庫多</t>
+  </si>
+  <si>
+    <t>CVE</t>
+  </si>
+  <si>
+    <t>中非法郎</t>
+  </si>
+  <si>
+    <t>XAF</t>
+  </si>
+  <si>
+    <t>西非法郎</t>
+  </si>
+  <si>
+    <t>XOF</t>
+  </si>
+  <si>
+    <t>加纳塞地</t>
+  </si>
+  <si>
+    <t>加納塞地</t>
+  </si>
+  <si>
+    <t>GHS</t>
+  </si>
+  <si>
+    <t>冈比亚达拉西</t>
+  </si>
+  <si>
+    <t>岡比亞達拉西</t>
+  </si>
+  <si>
+    <t>GMD</t>
+  </si>
+  <si>
+    <t>几内亚法郎</t>
+  </si>
+  <si>
+    <t>幾內亞法郎</t>
+  </si>
+  <si>
+    <t>GNF</t>
+  </si>
+  <si>
+    <t>莱索托洛蒂</t>
+  </si>
+  <si>
+    <t>萊索托洛蒂</t>
+  </si>
+  <si>
+    <t>LSL</t>
+  </si>
+  <si>
+    <t>利比里亚元</t>
+  </si>
+  <si>
+    <t>利比里亞元</t>
+  </si>
+  <si>
+    <t>LRD</t>
+  </si>
+  <si>
+    <t>利比亚第纳尔</t>
+  </si>
+  <si>
+    <t>利比亞第納爾</t>
+  </si>
+  <si>
+    <t>LYD</t>
+  </si>
+  <si>
+    <t>马达加斯加阿里亚里</t>
+  </si>
+  <si>
+    <t>馬達加斯加阿里亞里</t>
+  </si>
+  <si>
+    <t>MGA</t>
+  </si>
+  <si>
+    <t>马拉维克瓦查</t>
+  </si>
+  <si>
+    <t>馬拉維克瓦查</t>
+  </si>
+  <si>
+    <t>MWK</t>
+  </si>
+  <si>
+    <t>毛里塔尼亚乌吉亚</t>
+  </si>
+  <si>
+    <t>毛里塔尼亞烏吉亞</t>
+  </si>
+  <si>
+    <t>MRU</t>
+  </si>
+  <si>
+    <t>毛里求斯卢比</t>
+  </si>
+  <si>
+    <t>毛里求斯盧比</t>
+  </si>
+  <si>
+    <t>MUR</t>
+  </si>
+  <si>
+    <t>莫桑比克梅蒂卡尔</t>
+  </si>
+  <si>
+    <t>莫桑比克梅蒂卡爾</t>
+  </si>
+  <si>
+    <t>MZN</t>
+  </si>
+  <si>
+    <t>纳米比亚元</t>
+  </si>
+  <si>
+    <t>納米比亞元</t>
+  </si>
+  <si>
+    <t>NAD</t>
+  </si>
+  <si>
+    <t>卢旺达法郎</t>
+  </si>
+  <si>
+    <t>盧旺達法郎</t>
+  </si>
+  <si>
+    <t>RWF</t>
+  </si>
+  <si>
+    <t>圣多美和普林西比多布拉</t>
+  </si>
+  <si>
+    <t>聖多美和普林西比多布拉</t>
+  </si>
+  <si>
+    <t>STN</t>
+  </si>
+  <si>
+    <t>塞舌尔卢比</t>
+  </si>
+  <si>
+    <t>塞舌爾盧比</t>
+  </si>
+  <si>
+    <t>SCR</t>
+  </si>
+  <si>
+    <t>塞拉利昂利昂</t>
+  </si>
+  <si>
+    <t>SLE</t>
+  </si>
+  <si>
+    <t>索马里先令</t>
+  </si>
+  <si>
+    <t>索馬里先令</t>
+  </si>
+  <si>
+    <t>SOS</t>
+  </si>
+  <si>
+    <t>苏丹镑</t>
+  </si>
+  <si>
+    <t>蘇丹鎊</t>
+  </si>
+  <si>
+    <t>SDG</t>
+  </si>
+  <si>
+    <t>斯威士兰里兰吉尼</t>
+  </si>
+  <si>
+    <t>斯威士蘭里蘭吉尼</t>
+  </si>
+  <si>
+    <t>SZL</t>
+  </si>
+  <si>
+    <t>坦桑尼亚先令</t>
+  </si>
+  <si>
+    <t>坦桑尼亞先令</t>
+  </si>
+  <si>
+    <t>TZS</t>
+  </si>
+  <si>
+    <t>突尼斯第纳尔</t>
+  </si>
+  <si>
+    <t>突尼斯第納爾</t>
+  </si>
+  <si>
+    <t>TND</t>
+  </si>
+  <si>
+    <t>乌干达先令</t>
+  </si>
+  <si>
+    <t>烏干達先令</t>
+  </si>
+  <si>
+    <t>UGX</t>
+  </si>
+  <si>
+    <t>赞比亚克瓦查</t>
+  </si>
+  <si>
+    <t>贊比亞克瓦查</t>
+  </si>
+  <si>
+    <t>ZMW</t>
+  </si>
+  <si>
+    <t>津巴布韦元</t>
+  </si>
+  <si>
+    <t>津巴布韋元</t>
+  </si>
+  <si>
+    <t>ZWG</t>
+  </si>
+  <si>
+    <t>东加勒比元</t>
+  </si>
+  <si>
+    <t>東加勒比元</t>
+  </si>
+  <si>
+    <t>XCD</t>
+  </si>
+  <si>
+    <t>巴哈马元</t>
+  </si>
+  <si>
+    <t>巴哈馬元</t>
+  </si>
+  <si>
+    <t>BSD</t>
+  </si>
+  <si>
+    <t>巴巴多斯元</t>
+  </si>
+  <si>
+    <t>BBD</t>
+  </si>
+  <si>
+    <t>伯利兹元</t>
+  </si>
+  <si>
+    <t>伯利茲元</t>
+  </si>
+  <si>
+    <t>BZD</t>
+  </si>
+  <si>
+    <t>萨尔瓦多科朗</t>
+  </si>
+  <si>
+    <t>薩爾瓦多科朗</t>
+  </si>
+  <si>
+    <t>SVC</t>
+  </si>
+  <si>
+    <t>危地马拉格查尔</t>
+  </si>
+  <si>
+    <t>危地馬拉格查爾</t>
+  </si>
+  <si>
+    <t>GTQ</t>
+  </si>
+  <si>
+    <t>洪都拉斯伦皮拉</t>
+  </si>
+  <si>
+    <t>洪都拉斯倫皮拉</t>
+  </si>
+  <si>
+    <t>HNL</t>
+  </si>
+  <si>
+    <t>海地古德</t>
+  </si>
+  <si>
+    <t>HTG</t>
+  </si>
+  <si>
+    <t>牙买加元</t>
+  </si>
+  <si>
+    <t>牙買加元</t>
+  </si>
+  <si>
+    <t>JMD</t>
+  </si>
+  <si>
+    <t>尼加拉瓜奥多巴</t>
+  </si>
+  <si>
+    <t>尼加拉瓜奧多巴</t>
+  </si>
+  <si>
+    <t>NIO</t>
+  </si>
+  <si>
+    <t>巴拿马巴波亚</t>
+  </si>
+  <si>
+    <t>巴拿馬巴波亞</t>
+  </si>
+  <si>
+    <t>PAB</t>
+  </si>
+  <si>
+    <t>特立尼达和多巴哥元</t>
+  </si>
+  <si>
+    <t>特立尼達和多巴哥元</t>
+  </si>
+  <si>
+    <t>TTD</t>
+  </si>
+  <si>
+    <t>太平洋法郎</t>
+  </si>
+  <si>
+    <t>XPF</t>
+  </si>
+  <si>
+    <t>巴布亚新几内亚基那</t>
+  </si>
+  <si>
+    <t>巴布亞新幾內亞基那</t>
+  </si>
+  <si>
+    <t>PGK</t>
+  </si>
+  <si>
+    <t>萨摩亚塔拉</t>
+  </si>
+  <si>
+    <t>薩摩亞塔拉</t>
+  </si>
+  <si>
+    <t>WST</t>
+  </si>
+  <si>
+    <t>所罗门群岛元</t>
+  </si>
+  <si>
+    <t>所羅門群島元</t>
+  </si>
+  <si>
+    <t>SBD</t>
+  </si>
+  <si>
+    <t>汤加潘加</t>
+  </si>
+  <si>
+    <t>湯加潘加</t>
+  </si>
+  <si>
+    <t>TOP</t>
+  </si>
+  <si>
+    <t>瓦努阿图瓦图</t>
+  </si>
+  <si>
+    <t>瓦努阿圖瓦圖</t>
+  </si>
+  <si>
+    <t>VUV</t>
+  </si>
+  <si>
+    <t>马尔代夫拉菲亚</t>
+  </si>
+  <si>
+    <t>馬爾代夫拉菲亞</t>
+  </si>
+  <si>
+    <t>MVR</t>
+  </si>
+  <si>
+    <t>文莱元</t>
+  </si>
+  <si>
+    <t>文萊元</t>
+  </si>
+  <si>
+    <t>BND</t>
+  </si>
+  <si>
+    <t>不丹努尔特鲁姆</t>
+  </si>
+  <si>
+    <t>不丹努爾特魯姆</t>
+  </si>
+  <si>
+    <t>BTN</t>
+  </si>
+  <si>
+    <t>科摩罗法郎</t>
+  </si>
+  <si>
+    <t>科摩羅法郎</t>
+  </si>
+  <si>
+    <t>KMF</t>
+  </si>
+  <si>
+    <t>直布罗陀镑</t>
+  </si>
+  <si>
+    <t>直布羅陀鎊</t>
+  </si>
+  <si>
+    <t>GIP</t>
+  </si>
+  <si>
+    <t>福克兰群岛镑</t>
+  </si>
+  <si>
+    <t>福克蘭群島鎊</t>
+  </si>
+  <si>
+    <t>FKP</t>
+  </si>
+  <si>
+    <t>圣赫勒拿镑</t>
+  </si>
+  <si>
+    <t>聖赫勒拿鎊</t>
+  </si>
+  <si>
+    <t>SHP</t>
+  </si>
+  <si>
+    <t>阿鲁巴弗罗林</t>
+  </si>
+  <si>
+    <t>阿魯巴弗羅林</t>
+  </si>
+  <si>
+    <t>AWG</t>
+  </si>
+  <si>
+    <t>荷属安地列斯盾</t>
+  </si>
+  <si>
+    <t>荷屬安地列斯盾</t>
+  </si>
+  <si>
+    <t>ANG</t>
+  </si>
+  <si>
+    <t>开曼群岛元</t>
+  </si>
+  <si>
+    <t>開曼群島元</t>
+  </si>
+  <si>
+    <t>KYD</t>
+  </si>
+  <si>
+    <t>百慕大元</t>
+  </si>
+  <si>
+    <t>百慕達元</t>
+  </si>
+  <si>
+    <t>BMD</t>
+  </si>
+  <si>
+    <t>泽西岛镑</t>
+  </si>
+  <si>
+    <t>澤西島鎊</t>
+  </si>
+  <si>
+    <t>JEP</t>
+  </si>
+  <si>
+    <t>根西岛镑</t>
+  </si>
+  <si>
+    <t>根西島鎊</t>
+  </si>
+  <si>
+    <t>GGP</t>
+  </si>
+  <si>
+    <t>马恩岛镑</t>
+  </si>
+  <si>
+    <t>馬恩島鎊</t>
+  </si>
+  <si>
+    <t>IMP</t>
+  </si>
+  <si>
+    <t>法罗克朗</t>
+  </si>
+  <si>
+    <t>法羅克朗</t>
+  </si>
+  <si>
+    <t>FOK</t>
+  </si>
+  <si>
+    <t>库克群岛元</t>
+  </si>
+  <si>
+    <t>庫克群島元</t>
+  </si>
+  <si>
+    <t>CKD</t>
+  </si>
+  <si>
+    <t>比特币</t>
+  </si>
+  <si>
+    <t>比特幣</t>
+  </si>
+  <si>
+    <t>BTC</t>
+  </si>
+  <si>
+    <t>以太坊</t>
+  </si>
+  <si>
+    <t>ETH</t>
+  </si>
+  <si>
+    <t>泰达币</t>
+  </si>
+  <si>
+    <t>泰達幣</t>
+  </si>
+  <si>
+    <t>USDT</t>
+  </si>
+  <si>
+    <t>USDC</t>
+  </si>
+  <si>
+    <t>币安币</t>
+  </si>
+  <si>
+    <t>幣安幣</t>
+  </si>
+  <si>
+    <t>BNB</t>
+  </si>
+  <si>
+    <t>索拉纳</t>
+  </si>
+  <si>
+    <t>索拉納</t>
+  </si>
+  <si>
+    <t>SOL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="5">
+  <numFmts count="4">
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="176" formatCode="0.00_);[Red]\(0.00\)"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -488,11 +1333,6 @@
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <name val="宋体"/>
-      <charset val="134"/>
     </font>
     <font>
       <u/>
@@ -974,141 +1814,138 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1116,9 +1953,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1645,33 +2479,33 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F52"/>
-  <sheetFormatPr defaultColWidth="16.015625" defaultRowHeight="16.8" outlineLevelCol="5"/>
+  <dimension ref="A1:C152"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="5" width="16.015625" customWidth="1"/>
-    <col min="6" max="6" width="16.015625" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="16.015625" customWidth="1"/>
+    <col min="1" max="1" width="15.78125" customWidth="1"/>
+    <col min="2" max="2" width="22.125" customWidth="1"/>
+    <col min="3" max="3" width="21.609375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17.75" spans="1:3">
-      <c r="A1" s="2" t="s">
+    <row r="1" ht="34.75" spans="1:3">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" ht="17.75" spans="1:3">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1687,543 +2521,1642 @@
       </c>
     </row>
     <row r="4" ht="17.75" spans="1:3">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="5" ht="17.75" spans="1:3">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="6" ht="17.75" spans="1:3">
-      <c r="A6" s="3" t="s">
+    <row r="6" ht="34.75" spans="1:3">
+      <c r="A6" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="7" ht="17.75" spans="1:6">
-      <c r="A7" s="3" t="s">
+    <row r="7" ht="17.75" spans="1:3">
+      <c r="A7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="F7" s="4"/>
     </row>
     <row r="8" ht="17.75" spans="1:3">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="3" t="s">
+    </row>
+    <row r="9" ht="17.75" spans="1:3">
+      <c r="A9" s="2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="9" ht="17.75" spans="1:3">
-      <c r="A9" s="3" t="s">
+      <c r="B9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B9" s="3" t="s">
+    </row>
+    <row r="10" ht="17.75" spans="1:3">
+      <c r="A10" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="B10" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="10" ht="17.75" spans="1:3">
-      <c r="A10" s="3" t="s">
+    <row r="11" ht="17.75" spans="1:3">
+      <c r="A11" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B11" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C10" s="3" t="s">
+    </row>
+    <row r="12" ht="17.75" spans="1:3">
+      <c r="A12" s="2" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="11" ht="17.75" spans="1:3">
-      <c r="A11" s="3" t="s">
+      <c r="B12" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B11" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C11" s="3" t="s">
+    </row>
+    <row r="13" ht="17.75" spans="1:3">
+      <c r="A13" s="2" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="12" ht="34.75" spans="1:3">
-      <c r="A12" s="3" t="s">
+      <c r="B13" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="C13" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C12" s="3" t="s">
+    </row>
+    <row r="14" ht="17.75" spans="1:3">
+      <c r="A14" s="2" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="13" ht="34.75" spans="1:3">
-      <c r="A13" s="3" t="s">
+      <c r="B14" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="C14" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C13" s="3" t="s">
+    </row>
+    <row r="15" ht="34.75" spans="1:3">
+      <c r="A15" s="2" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="14" ht="17.75" spans="1:3">
-      <c r="A14" s="3" t="s">
+      <c r="B15" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="C15" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C14" s="3" t="s">
+    </row>
+    <row r="16" ht="17.75" spans="1:3">
+      <c r="A16" s="2" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="15" ht="17.75" spans="1:3">
-      <c r="A15" s="3" t="s">
+      <c r="B16" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="C16" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C15" s="3" t="s">
+    </row>
+    <row r="17" ht="17.75" spans="1:3">
+      <c r="A17" s="2" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="16" ht="17.75" spans="1:3">
-      <c r="A16" s="3" t="s">
+      <c r="B17" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B16" s="3" t="s">
+    </row>
+    <row r="18" ht="17.75" spans="1:3">
+      <c r="A18" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="B18" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="17" ht="34.75" spans="1:3">
-      <c r="A17" s="3" t="s">
+    <row r="19" ht="17.75" spans="1:3">
+      <c r="A19" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B19" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C19" s="2" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="18" ht="17.75" spans="1:3">
-      <c r="A18" s="3" t="s">
+    <row r="20" ht="17.75" spans="1:3">
+      <c r="A20" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B20" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C20" s="2" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="19" ht="17.75" spans="1:3">
-      <c r="A19" s="3" t="s">
+    <row r="21" ht="17.75" spans="1:3">
+      <c r="A21" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B21" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C21" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="20" ht="34.75" spans="1:3">
-      <c r="A20" s="3" t="s">
+    <row r="22" ht="34.75" spans="1:3">
+      <c r="A22" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B22" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C22" s="2" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="21" ht="17.75" spans="1:3">
-      <c r="A21" s="3" t="s">
+    <row r="23" ht="17.75" spans="1:3">
+      <c r="A23" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B23" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C23" s="2" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="22" ht="34.75" spans="1:3">
-      <c r="A22" s="3" t="s">
+    <row r="24" ht="34.75" spans="1:3">
+      <c r="A24" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B24" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="C24" s="2" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="23" ht="17.75" spans="1:3">
-      <c r="A23" s="3" t="s">
+    <row r="25" ht="17.75" spans="1:3">
+      <c r="A25" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B25" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C25" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="24" ht="34.75" spans="1:3">
-      <c r="A24" s="3" t="s">
+    <row r="26" ht="17.75" spans="1:3">
+      <c r="A26" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B26" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="C26" s="2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="25" ht="17.75" spans="1:3">
-      <c r="A25" s="3" t="s">
+    <row r="27" ht="34.75" spans="1:3">
+      <c r="A27" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B27" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="C27" s="2" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="26" ht="34.75" spans="1:3">
-      <c r="A26" s="3" t="s">
+    <row r="28" ht="34.75" spans="1:3">
+      <c r="A28" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B26" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="C26" s="3" t="s">
+      <c r="B28" s="2" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="27" ht="17.75" spans="1:3">
-      <c r="A27" s="3" t="s">
+      <c r="C28" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="B27" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="C27" s="3" t="s">
+    </row>
+    <row r="29" ht="34.75" spans="1:3">
+      <c r="A29" s="2" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="28" ht="17.75" spans="1:3">
-      <c r="A28" s="3" t="s">
+      <c r="B29" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B28" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="C28" s="3" t="s">
+      <c r="C29" s="2" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="29" ht="17.75" spans="1:3">
-      <c r="A29" s="3" t="s">
+    <row r="30" ht="34.75" spans="1:3">
+      <c r="A30" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="B30" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C30" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="C29" s="3" t="s">
+    </row>
+    <row r="31" ht="17.75" spans="1:3">
+      <c r="A31" s="2" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="30" ht="34.75" spans="1:3">
-      <c r="A30" s="3" t="s">
+      <c r="B31" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="B30" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="C30" s="3" t="s">
+      <c r="C31" s="2" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="31" ht="34.75" spans="1:3">
-      <c r="A31" s="3" t="s">
+    <row r="32" ht="34.75" spans="1:3">
+      <c r="A32" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B31" s="3" t="s">
+      <c r="B32" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C31" s="3" t="s">
+      <c r="C32" s="2" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="32" ht="34.75" spans="1:3">
-      <c r="A32" s="3" t="s">
+    <row r="33" ht="34.75" spans="1:3">
+      <c r="A33" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="B33" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="C32" s="3" t="s">
+      <c r="C33" s="2" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="33" ht="34.75" spans="1:3">
-      <c r="A33" s="3" t="s">
+    <row r="34" ht="34.75" spans="1:3">
+      <c r="A34" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="B33" s="3" t="s">
+      <c r="B34" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="C33" s="3" t="s">
+      <c r="C34" s="2" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="34" ht="34.75" spans="1:3">
-      <c r="A34" s="3" t="s">
+    <row r="35" ht="34.75" spans="1:3">
+      <c r="A35" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B34" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="C34" s="3" t="s">
+      <c r="B35" s="2" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="35" ht="17.75" spans="1:3">
-      <c r="A35" s="3" t="s">
+      <c r="C35" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B35" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="C35" s="3" t="s">
+    </row>
+    <row r="36" ht="34.75" spans="1:3">
+      <c r="A36" s="2" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="36" ht="34.75" spans="1:3">
-      <c r="A36" s="3" t="s">
+      <c r="B36" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="B36" s="3" t="s">
+      <c r="C36" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="C36" s="3" t="s">
+    </row>
+    <row r="37" ht="34.75" spans="1:3">
+      <c r="A37" s="2" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="37" ht="17.75" spans="1:3">
-      <c r="A37" s="3" t="s">
+      <c r="B37" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C37" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="B37" s="3" t="s">
+    </row>
+    <row r="38" ht="34.75" spans="1:3">
+      <c r="A38" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C37" s="3" t="s">
+      <c r="B38" s="2" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="38" ht="17.75" spans="1:3">
-      <c r="A38" s="3" t="s">
+      <c r="C38" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="B38" s="3" t="s">
+    </row>
+    <row r="39" ht="17.75" spans="1:3">
+      <c r="A39" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="C38" s="3" t="s">
+      <c r="B39" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="C39" s="2" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="39" ht="34.75" spans="1:3">
-      <c r="A39" s="3" t="s">
+    <row r="40" ht="34.75" spans="1:3">
+      <c r="A40" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B39" s="3" t="s">
+      <c r="B40" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="C39" s="3" t="s">
+      <c r="C40" s="2" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="40" ht="34.75" spans="1:3">
-      <c r="A40" s="3" t="s">
+    <row r="41" ht="34.75" spans="1:3">
+      <c r="A41" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="B40" s="3" t="s">
+      <c r="B41" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C40" s="3" t="s">
+      <c r="C41" s="2" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="41" ht="17.75" spans="1:3">
-      <c r="A41" s="3" t="s">
+    <row r="42" ht="34.75" spans="1:3">
+      <c r="A42" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="B41" s="3" t="s">
+      <c r="B42" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="C41" s="3" t="s">
+      <c r="C42" s="2" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="42" ht="34.75" spans="1:3">
-      <c r="A42" s="3" t="s">
+    <row r="43" ht="17.75" spans="1:3">
+      <c r="A43" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="B42" s="3" t="s">
+      <c r="B43" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C43" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="C42" s="3" t="s">
+    </row>
+    <row r="44" ht="34.75" spans="1:3">
+      <c r="A44" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="43" ht="34.75" spans="1:3">
-      <c r="A43" s="3" t="s">
+      <c r="B44" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="B43" s="3" t="s">
+      <c r="C44" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="C43" s="3" t="s">
+    </row>
+    <row r="45" ht="17.75" spans="1:3">
+      <c r="A45" s="2" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="44" ht="34.75" spans="1:3">
-      <c r="A44" s="3" t="s">
+      <c r="B45" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="B44" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="C44" s="3" t="s">
+      <c r="C45" s="2" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="45" ht="34.75" spans="1:3">
-      <c r="A45" s="3" t="s">
+    <row r="46" ht="34.75" spans="1:3">
+      <c r="A46" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="B45" s="3" t="s">
+      <c r="B46" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="C45" s="3" t="s">
+      <c r="C46" s="2" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="46" ht="34.75" spans="1:3">
-      <c r="A46" s="3" t="s">
+    <row r="47" ht="34.75" spans="1:3">
+      <c r="A47" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="B46" s="3" t="s">
+      <c r="B47" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="C46" s="3" t="s">
+      <c r="C47" s="2" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="47" ht="34.75" spans="1:3">
-      <c r="A47" s="3" t="s">
+    <row r="48" ht="34.75" spans="1:3">
+      <c r="A48" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="B47" s="3" t="s">
+      <c r="B48" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="C47" s="3" t="s">
+      <c r="C48" s="2" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="48" ht="34.75" spans="1:3">
-      <c r="A48" s="3" t="s">
+    <row r="49" ht="17.75" spans="1:3">
+      <c r="A49" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="B48" s="3" t="s">
+      <c r="B49" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="C48" s="3" t="s">
+      <c r="C49" s="2" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="49" ht="34.75" spans="1:3">
-      <c r="A49" s="3" t="s">
+    <row r="50" ht="34.75" spans="1:3">
+      <c r="A50" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="B49" s="3" t="s">
+      <c r="B50" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="C50" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="C49" s="3" t="s">
+    </row>
+    <row r="51" ht="17.75" spans="1:3">
+      <c r="A51" s="2" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="50" ht="34.75" spans="1:3">
-      <c r="A50" s="3" t="s">
+      <c r="B51" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="B50" s="3" t="s">
+      <c r="C51" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="C50" s="3" t="s">
+    </row>
+    <row r="52" ht="34.75" spans="1:3">
+      <c r="A52" s="2" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="51" ht="34.75" spans="1:3">
-      <c r="A51" s="3" t="s">
+      <c r="B52" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="B51" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="C51" s="3" t="s">
+      <c r="C52" s="2" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="52" ht="17.75" spans="1:3">
-      <c r="A52" s="3" t="s">
+    <row r="53" ht="34.75" spans="1:3">
+      <c r="A53" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="B52" s="3" t="s">
+      <c r="B53" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="C52" s="3" t="s">
+      <c r="C53" s="2" t="s">
         <v>141</v>
+      </c>
+    </row>
+    <row r="54" ht="34.75" spans="1:3">
+      <c r="A54" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="55" ht="34.75" spans="1:3">
+      <c r="A55" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="56" ht="34.75" spans="1:3">
+      <c r="A56" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="57" ht="17.75" spans="1:3">
+      <c r="A57" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="58" ht="34.75" spans="1:3">
+      <c r="A58" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="59" ht="34.75" spans="1:3">
+      <c r="A59" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="60" ht="34.75" spans="1:3">
+      <c r="A60" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="61" ht="34.75" spans="1:3">
+      <c r="A61" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="62" ht="34.75" spans="1:3">
+      <c r="A62" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="63" ht="34.75" spans="1:3">
+      <c r="A63" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="64" ht="34.75" spans="1:3">
+      <c r="A64" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="65" ht="34.75" spans="1:3">
+      <c r="A65" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="66" ht="34.75" spans="1:3">
+      <c r="A66" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="67" ht="34.75" spans="1:3">
+      <c r="A67" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="68" ht="34.75" spans="1:3">
+      <c r="A68" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="69" ht="34.75" spans="1:3">
+      <c r="A69" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="70" ht="34.75" spans="1:3">
+      <c r="A70" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="71" ht="34.75" spans="1:3">
+      <c r="A71" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="72" ht="34.75" spans="1:3">
+      <c r="A72" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="73" ht="34.75" spans="1:3">
+      <c r="A73" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="74" ht="34.75" spans="1:3">
+      <c r="A74" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="75" ht="17.75" spans="1:3">
+      <c r="A75" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="76" ht="17.75" spans="1:3">
+      <c r="A76" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="77" ht="17.75" spans="1:3">
+      <c r="A77" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="78" ht="34.75" spans="1:3">
+      <c r="A78" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="79" ht="34.75" spans="1:3">
+      <c r="A79" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="80" ht="34.75" spans="1:3">
+      <c r="A80" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="81" ht="34.75" spans="1:3">
+      <c r="A81" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="C81" s="2" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="82" ht="34.75" spans="1:3">
+      <c r="A82" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="C82" s="2" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="83" ht="34.75" spans="1:3">
+      <c r="A83" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="84" ht="17.75" spans="1:3">
+      <c r="A84" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="85" ht="34.75" spans="1:3">
+      <c r="A85" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="86" ht="34.75" spans="1:3">
+      <c r="A86" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="87" ht="17.75" spans="1:3">
+      <c r="A87" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="C87" s="2" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="88" ht="17.75" spans="1:3">
+      <c r="A88" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="C88" s="2" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="89" ht="17.75" spans="1:3">
+      <c r="A89" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="90" ht="34.75" spans="1:3">
+      <c r="A90" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="C90" s="2" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="91" ht="34.75" spans="1:3">
+      <c r="A91" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="B91" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="C91" s="2" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="92" ht="34.75" spans="1:3">
+      <c r="A92" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="B92" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="C92" s="2" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="93" ht="34.75" spans="1:3">
+      <c r="A93" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="B93" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="C93" s="2" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="94" ht="34.75" spans="1:3">
+      <c r="A94" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="B94" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="C94" s="2" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="95" ht="51.75" spans="1:3">
+      <c r="A95" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="96" ht="34.75" spans="1:3">
+      <c r="A96" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="B96" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="C96" s="2" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="97" ht="34.75" spans="1:3">
+      <c r="A97" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="C97" s="2" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="98" ht="34.75" spans="1:3">
+      <c r="A98" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="B98" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="99" ht="34.75" spans="1:3">
+      <c r="A99" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="B99" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="100" ht="34.75" spans="1:3">
+      <c r="A100" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="B100" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="C100" s="2" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="101" ht="34.75" spans="1:3">
+      <c r="A101" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="B101" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="C101" s="2" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="102" ht="51.75" spans="1:3">
+      <c r="A102" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="103" ht="34.75" spans="1:3">
+      <c r="A103" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="B103" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="C103" s="2" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="104" ht="34.75" spans="1:3">
+      <c r="A104" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="B104" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="105" ht="34.75" spans="1:3">
+      <c r="A105" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="B105" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="C105" s="2" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="106" ht="17.75" spans="1:3">
+      <c r="A106" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="B106" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="C106" s="2" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="107" ht="34.75" spans="1:3">
+      <c r="A107" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="B107" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="C107" s="2" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="108" ht="34.75" spans="1:3">
+      <c r="A108" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="B108" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="C108" s="2" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="109" ht="34.75" spans="1:3">
+      <c r="A109" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="B109" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="C109" s="2" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="110" ht="34.75" spans="1:3">
+      <c r="A110" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="B110" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="C110" s="2" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="111" ht="34.75" spans="1:3">
+      <c r="A111" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="B111" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="C111" s="2" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="112" ht="34.75" spans="1:3">
+      <c r="A112" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="B112" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="C112" s="2" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="113" ht="34.75" spans="1:3">
+      <c r="A113" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="B113" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="C113" s="2" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="114" ht="17.75" spans="1:3">
+      <c r="A114" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="B114" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="C114" s="2" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="115" ht="34.75" spans="1:3">
+      <c r="A115" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="B115" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="C115" s="2" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="116" ht="17.75" spans="1:3">
+      <c r="A116" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="B116" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="C116" s="2" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="117" ht="34.75" spans="1:3">
+      <c r="A117" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="B117" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="C117" s="2" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="118" ht="34.75" spans="1:3">
+      <c r="A118" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="B118" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="C118" s="2" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="119" ht="34.75" spans="1:3">
+      <c r="A119" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="B119" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="C119" s="2" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="120" ht="17.75" spans="1:3">
+      <c r="A120" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="B120" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="C120" s="2" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="121" ht="17.75" spans="1:3">
+      <c r="A121" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="B121" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="C121" s="2" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="122" ht="34.75" spans="1:3">
+      <c r="A122" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="B122" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="C122" s="2" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="123" ht="34.75" spans="1:3">
+      <c r="A123" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="B123" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="C123" s="2" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="124" ht="51.75" spans="1:3">
+      <c r="A124" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="B124" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="C124" s="2" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="125" ht="34.75" spans="1:3">
+      <c r="A125" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="B125" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="C125" s="2" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="126" ht="51.75" spans="1:3">
+      <c r="A126" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="B126" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="C126" s="2" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="127" ht="34.75" spans="1:3">
+      <c r="A127" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="B127" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="C127" s="2" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="128" ht="34.75" spans="1:3">
+      <c r="A128" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="B128" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="C128" s="2" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="129" ht="17.75" spans="1:3">
+      <c r="A129" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="B129" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="C129" s="2" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="130" ht="34.75" spans="1:3">
+      <c r="A130" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="B130" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="C130" s="2" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="131" ht="34.75" spans="1:3">
+      <c r="A131" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="B131" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="C131" s="2" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="132" ht="17.75" spans="1:3">
+      <c r="A132" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="B132" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="C132" s="2" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="133" ht="34.75" spans="1:3">
+      <c r="A133" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="B133" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="C133" s="2" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="134" ht="34.75" spans="1:3">
+      <c r="A134" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="B134" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="C134" s="2" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="135" ht="34.75" spans="1:3">
+      <c r="A135" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="B135" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="C135" s="2" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="136" ht="34.75" spans="1:3">
+      <c r="A136" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="B136" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="C136" s="2" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="137" ht="34.75" spans="1:3">
+      <c r="A137" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="B137" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="C137" s="2" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="138" ht="34.75" spans="1:3">
+      <c r="A138" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="B138" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="C138" s="2" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="139" ht="34.75" spans="1:3">
+      <c r="A139" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="B139" s="2" t="s">
+        <v>386</v>
+      </c>
+      <c r="C139" s="2" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="140" ht="34.75" spans="1:3">
+      <c r="A140" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="B140" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="C140" s="2" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="141" ht="17.75" spans="1:3">
+      <c r="A141" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="B141" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="C141" s="2" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="142" ht="17.75" spans="1:3">
+      <c r="A142" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="B142" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="C142" s="2" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="143" ht="17.75" spans="1:3">
+      <c r="A143" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="B143" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="C143" s="2" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="144" ht="17.75" spans="1:3">
+      <c r="A144" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="B144" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="C144" s="2" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="145" ht="17.75" spans="1:3">
+      <c r="A145" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="B145" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="C145" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="146" ht="34.75" spans="1:3">
+      <c r="A146" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="B146" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="C146" s="2" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="147" ht="17.75" spans="1:3">
+      <c r="A147" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="B147" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="C147" s="2" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="148" ht="17.75" spans="1:3">
+      <c r="A148" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="B148" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="C148" s="2" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="149" ht="17.75" spans="1:3">
+      <c r="A149" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="B149" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="C149" s="2" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="150" ht="17.75" spans="1:3">
+      <c r="A150" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="B150" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="C150" s="2" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="151" ht="17.75" spans="1:3">
+      <c r="A151" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="B151" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="C151" s="2" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="152" ht="17.75" spans="1:3">
+      <c r="A152" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="B152" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="C152" s="2" t="s">
+        <v>423</v>
       </c>
     </row>
   </sheetData>

</xml_diff>